<commit_message>
auto: update toolset portal
</commit_message>
<xml_diff>
--- a/AI 工具集.xlsx
+++ b/AI 工具集.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21710" windowHeight="10910"/>
+    <workbookView windowWidth="22560" windowHeight="10910"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
   <si>
     <t>自建网页</t>
   </si>
@@ -85,69 +85,33 @@
     <t>https://mightymojoy.github.io/douyin_dashboard/</t>
   </si>
   <si>
-    <t>内容短视频数据看板</t>
-  </si>
-  <si>
-    <t>https://mightymojoy.github.io/Content-short-video/</t>
-  </si>
-  <si>
-    <t>ITO内容生成摄影提示词</t>
-  </si>
-  <si>
-    <t>https://mightymojoy.github.io/photography-prompt/</t>
+    <t>ITO内容短视频脚本生成器</t>
+  </si>
+  <si>
+    <t>https://mightymojoy.github.io/NEW-DY-short-videos/</t>
   </si>
   <si>
     <t>内容创作工具</t>
   </si>
   <si>
-    <t>ITO内容短视频脚本生成器</t>
-  </si>
-  <si>
-    <t>https://mightymojoy.github.io/NEW-DY-short-videos/</t>
-  </si>
-  <si>
     <t>ITO摄影提示词精准控制生成</t>
   </si>
   <si>
     <t>https://mightymojoy.github.io/ITO-PROMPT-STUDIO/ITO-Prompt-Studio.html</t>
   </si>
   <si>
-    <t>内容排版助手</t>
-  </si>
-  <si>
-    <t>https://layout-beta-lyart.vercel.app/</t>
-  </si>
-  <si>
     <t>ITO新品介绍</t>
   </si>
   <si>
     <t>https://itonewproduct.vercel.app/</t>
   </si>
   <si>
-    <t>ITO AI 考试智能评分</t>
-  </si>
-  <si>
-    <t>https://ito-ai-grading.vercel.app/</t>
-  </si>
-  <si>
     <t>ITO FCST预测（待完善）</t>
   </si>
   <si>
     <t>https://mightymojoy.github.io/fcst_dashboard/</t>
   </si>
   <si>
-    <t>ITO 提示词-基础操作-职场版</t>
-  </si>
-  <si>
-    <t>https://mightymojoy.github.io/PROMPT/</t>
-  </si>
-  <si>
-    <t>AI 自建小工具</t>
-  </si>
-  <si>
-    <t>https://mightymojoy.github.io/AI-WORKSHOP/ITO_AI%E5%B7%A5%E4%BD%9C%E5%9D%8A_%E5%AD%A6%E5%91%98%E7%89%88.html</t>
-  </si>
-  <si>
     <t>京东毛保监控</t>
   </si>
   <si>
@@ -166,7 +130,7 @@
     <t>https://www.htmlcode.fun/s/yg8par7a</t>
   </si>
   <si>
-    <t>ITO AI EGENT 测试</t>
+    <t>ITO AI AGENT 测试</t>
   </si>
   <si>
     <t xml:space="preserve">https://ito-ai-grading.vercel.app/agent-exam.html      </t>
@@ -1153,7 +1117,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1251,18 +1215,18 @@
         <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
         <v>20</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1273,7 +1237,7 @@
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1284,7 +1248,7 @@
         <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1295,7 +1259,7 @@
         <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1306,7 +1270,7 @@
         <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1328,139 +1292,73 @@
         <v>34</v>
       </c>
       <c r="C16" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" t="s">
+      <c r="B17" s="2"/>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="B18" s="2"/>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>39</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C22" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C26" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C27" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
-        <v>53</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C28" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="A29" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>50</v>
+      <c r="C24" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1471,25 +1369,19 @@
     <hyperlink ref="B6" r:id="rId4" display="https://mightymojoy.github.io/live-dashboard/index.html"/>
     <hyperlink ref="B7" r:id="rId5" display="https://mightymojoy.github.io/live-dashboard/trend.html"/>
     <hyperlink ref="B8" r:id="rId6" display="https://mightymojoy.github.io/douyin_dashboard/"/>
-    <hyperlink ref="B9" r:id="rId7" display="https://mightymojoy.github.io/Content-short-video/"/>
-    <hyperlink ref="B10" r:id="rId8" display="https://mightymojoy.github.io/photography-prompt/"/>
-    <hyperlink ref="B11" r:id="rId9" display="https://mightymojoy.github.io/NEW-DY-short-videos/" tooltip="https://mightymojoy.github.io/NEW-DY-short-videos/"/>
-    <hyperlink ref="B12" r:id="rId10" display="https://mightymojoy.github.io/ITO-PROMPT-STUDIO/ITO-Prompt-Studio.html"/>
-    <hyperlink ref="B13" r:id="rId11" display="https://layout-beta-lyart.vercel.app/"/>
-    <hyperlink ref="B14" r:id="rId12" display="https://itonewproduct.vercel.app/"/>
-    <hyperlink ref="B15" r:id="rId13" display="https://ito-ai-grading.vercel.app/"/>
-    <hyperlink ref="B16" r:id="rId14" display="https://mightymojoy.github.io/fcst_dashboard/"/>
-    <hyperlink ref="B17" r:id="rId15" display="https://mightymojoy.github.io/PROMPT/"/>
-    <hyperlink ref="B26" r:id="rId16" display="https://my.feishu.cn/wiki/CgBmw84OSikaKZk0jImckrNjnug?sheet=kGV1ky"/>
-    <hyperlink ref="B27" r:id="rId17" display="https://my.feishu.cn/wiki/W6vewSdagixfhOkNqA0cAWtPn2e?sheet=iC9wkH"/>
-    <hyperlink ref="B28" r:id="rId18" display="https://my.feishu.cn/sheets/CtZuseYAyhrJPgtGBxFc755Vnge?sheet=JOlwMJ"/>
-    <hyperlink ref="B29" r:id="rId19" display="https://my.feishu.cn/sheets/RKudsmnm3h2cOPtvv4ScTEzSnCh"/>
-    <hyperlink ref="B18" r:id="rId20" display="https://mightymojoy.github.io/AI-WORKSHOP/ITO_AI%E5%B7%A5%E4%BD%9C%E5%9D%8A_%E5%AD%A6%E5%91%98%E7%89%88.html"/>
-    <hyperlink ref="B19" r:id="rId21" display="https://66396c5698674ebe9ee8a78092ef1298.app.codebuddy.work/"/>
-    <hyperlink ref="B20" r:id="rId22" display="https://metabase.doris.itocases.com/question/81?trade_time=2026-07&amp;shop_no=01"/>
-    <hyperlink ref="B30" r:id="rId23" display="https://my.feishu.cn/wiki/QWb6wpxXAiBjsjk3o9Qc98HunNe?table=tbljqLJy1V5S4cFP&amp;view=vewfJNQRH2#CategoryAutomatedNotification"/>
-    <hyperlink ref="B21" r:id="rId24" display="https://www.htmlcode.fun/s/yg8par7a"/>
-    <hyperlink ref="B22" r:id="rId25" display="https://ito-ai-grading.vercel.app/agent-exam.html      "/>
+    <hyperlink ref="B9" r:id="rId7" display="https://mightymojoy.github.io/NEW-DY-short-videos/" tooltip="https://mightymojoy.github.io/NEW-DY-short-videos/"/>
+    <hyperlink ref="B10" r:id="rId8" display="https://mightymojoy.github.io/ITO-PROMPT-STUDIO/ITO-Prompt-Studio.html"/>
+    <hyperlink ref="B11" r:id="rId9" display="https://itonewproduct.vercel.app/"/>
+    <hyperlink ref="B12" r:id="rId10" display="https://mightymojoy.github.io/fcst_dashboard/"/>
+    <hyperlink ref="B20" r:id="rId11" display="https://my.feishu.cn/wiki/CgBmw84OSikaKZk0jImckrNjnug?sheet=kGV1ky"/>
+    <hyperlink ref="B21" r:id="rId12" display="https://my.feishu.cn/wiki/W6vewSdagixfhOkNqA0cAWtPn2e?sheet=iC9wkH"/>
+    <hyperlink ref="B22" r:id="rId13" display="https://my.feishu.cn/sheets/CtZuseYAyhrJPgtGBxFc755Vnge?sheet=JOlwMJ"/>
+    <hyperlink ref="B23" r:id="rId14" display="https://my.feishu.cn/sheets/RKudsmnm3h2cOPtvv4ScTEzSnCh"/>
+    <hyperlink ref="B13" r:id="rId15" display="https://66396c5698674ebe9ee8a78092ef1298.app.codebuddy.work/"/>
+    <hyperlink ref="B14" r:id="rId16" display="https://metabase.doris.itocases.com/question/81?trade_time=2026-07&amp;shop_no=01"/>
+    <hyperlink ref="B24" r:id="rId17" display="https://my.feishu.cn/wiki/QWb6wpxXAiBjsjk3o9Qc98HunNe?table=tbljqLJy1V5S4cFP&amp;view=vewfJNQRH2#CategoryAutomatedNotification"/>
+    <hyperlink ref="B15" r:id="rId18" display="https://www.htmlcode.fun/s/yg8par7a"/>
+    <hyperlink ref="B16" r:id="rId19" display="https://ito-ai-grading.vercel.app/agent-exam.html      "/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>